<commit_message>
Tentativa de DistanciaEdicao - deve-se terminar ainda
</commit_message>
<xml_diff>
--- a/Pasta1.xlsx
+++ b/Pasta1.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.ferreira002\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Windows\Users\henri\Desktop\pucrs\5 sem\proj. e otim. de alg\6---problema-da-mochila-lucio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBF7B256-153D-44BE-82FA-6F87C0969167}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359C57EF-A9F7-4100-AEF8-22A2C9692B3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="9525" xr2:uid="{E302910E-6A11-4113-BF2E-F214013B0BC2}"/>
+    <workbookView xWindow="1092" yWindow="-108" windowWidth="22056" windowHeight="13176" xr2:uid="{E302910E-6A11-4113-BF2E-F214013B0BC2}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
   <si>
     <t>Recursivo</t>
   </si>
@@ -103,6 +103,12 @@
   </si>
   <si>
     <t>9;28</t>
+  </si>
+  <si>
+    <t>DistanciaEdicao</t>
+  </si>
+  <si>
+    <t>DistanciaEdicaoDinamica</t>
   </si>
 </sst>
 </file>
@@ -138,9 +144,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -159,7 +168,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -455,17 +464,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42407E0D-38FA-4736-A374-4B51FA833A81}">
-  <dimension ref="D3:K10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="D3:K13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="20.140625" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" customWidth="1"/>
+    <col min="4" max="4" width="22.44140625" customWidth="1"/>
+    <col min="8" max="8" width="16.109375" customWidth="1"/>
     <col min="9" max="9" width="30" customWidth="1"/>
-    <col min="10" max="10" width="43.5703125" customWidth="1"/>
-    <col min="11" max="11" width="28.28515625" customWidth="1"/>
+    <col min="10" max="10" width="43.5546875" customWidth="1"/>
+    <col min="11" max="11" width="28.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D3" t="s">
         <v>3</v>
       </c>
@@ -491,7 +500,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="4" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D4" t="s">
         <v>0</v>
       </c>
@@ -517,7 +526,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D5" t="s">
         <v>1</v>
       </c>
@@ -543,7 +552,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D6" t="s">
         <v>2</v>
       </c>
@@ -569,7 +578,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D9" t="s">
         <v>22</v>
       </c>
@@ -577,12 +586,25 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D10" t="s">
         <v>24</v>
       </c>
       <c r="E10" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="2">
+        <v>226572</v>
       </c>
     </row>
   </sheetData>

</xml_diff>